<commit_message>
Update workspace_history.xlsx with Day 2 project details
</commit_message>
<xml_diff>
--- a/workspace_history.xlsx
+++ b/workspace_history.xlsx
@@ -1,79 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Saurav\TTS\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B591AB0B-6E06-4D0B-A0AA-815DEE661BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Day</t>
-  </si>
-  <si>
-    <t>Phase</t>
-  </si>
-  <si>
-    <t>Tasks Completed</t>
-  </si>
-  <si>
-    <t>Key Deliverables</t>
-  </si>
-  <si>
-    <t>Day 1</t>
-  </si>
-  <si>
-    <t>1. Sourced and inspected 8 TTS models (Chatterbox Turbo, Fish Speech S2, XTTS-v2, CosyVoice 3, OmniVoice, IndexTTS2, Kokoro-82M, and ElevenLabs baseline).
-2. Generated initial comparison metrics (Inference Time, CPU/VRAM usage, Real-Time Factor) and created charts.
-3. Upgraded fallback speech engine from robotic Windows SAPI5 to highly natural neural backend (Kokoro-82M).
-4. Configured Streamlit thread-safety by wrapping CoInitialize calls for background execution.
-5. Integrated F5-TTS flow-matching zero-shot cloning to generate speech in your exact voice using my_voice.wav.
-6. Configured imageio-ffmpeg dynamically to bypass system-level FFmpeg path installation errors.
-7. Installed CUDA PyTorch to enable GPU acceleration, reducing cloning times from 152s (CPU) down to 5.2s (GPU) on RTX 3060.
-8. Created showcase.html, a fully self-contained sharing page with Base64 embedded audio files.</t>
-  </si>
-  <si>
-    <t>dashboard.py, scripts/speech_synth_helper.py, benchmark_results.csv, showcase.html, voices/my_voice.wav</t>
-  </si>
-  <si>
-    <t>TTS  Research, Benchmarking &amp; Custom Zero-Shot Voice Cloning</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -88,49 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -418,56 +420,93 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="63.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="161.77734375" customWidth="1"/>
-    <col min="4" max="4" width="91.5546875" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tasks Completed</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Key Deliverables</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TTS Laboratory Research, Benchmarking &amp; Custom Zero-Shot Voice Cloning</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1. Sourced and inspected 8 TTS models (Chatterbox Turbo, Fish Speech S2, XTTS-v2, CosyVoice 3, OmniVoice, IndexTTS2, Kokoro-82M, and ElevenLabs baseline).
+2. Generated initial comparison metrics (Inference Time, CPU/VRAM usage, Real-Time Factor) and created charts.
+3. Upgraded fallback speech engine from robotic Windows SAPI5 to highly natural neural backend (Kokoro-82M).
+4. Configured Streamlit thread-safety by wrapping CoInitialize calls for background execution.
+5. Integrated F5-TTS flow-matching zero-shot cloning to generate speech in your exact voice using my_voice.wav.
+6. Configured imageio-ffmpeg dynamically to bypass system-level FFmpeg path installation errors.
+7. Installed CUDA PyTorch to enable GPU acceleration, reducing cloning times from 152s (CPU) down to 5.2s (GPU) on RTX 3060.
+8. Created showcase.html, a fully self-contained sharing page with Base64 embedded audio files.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>dashboard.py, scripts/speech_synth_helper.py, benchmark_results.csv, showcase.html, voices/my_voice.wav</t>
+        </is>
+      </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="F7" s="3"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Local Model Storage, Voice Sample Cleaning, Pronunciation Engine, &amp; UI Studio Enhancements</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1. Integrated Audio8-TTS-Preview-0.6b, a dual autoregressive multilingual zero-shot voice cloning model.
+2. Implemented custom transformers class registration mapping in scripts/audio8/ to resolve HuggingFace dynamic package import issues on Windows.
+3. Cleaned background noise from user MP3 voice sample using noisereduce, converted to WAV, transcribed with Whisper for naming (that_feeling_of_being.wav), and trimmed to 40.0s.
+4. Migrated HuggingFace weights cache (Kokoro, F5-TTS, Vocos, Whisper, Audio8) from global C: drive to local virtual environment (.venv/hf_cache) and set HF_HOME redirection.
+5. Filtered non-critical Python warnings (Google, Torchaudio, PyTorch) and muted HuggingFace HTTP HEAD connection retries in the console logs.
+6. Added interactive Voice Tuning post-processing sliders (Pitch shift, Speed/Tempo stretch, Audio Trimming) using librosa's phase vocoder.
+7. Designed the Voice Clone Arena comparison tab, enabling side-by-side prompt synthesis and latency metrics across multiple engines in columns.
+8. Createdconfigs/pronunciation_map.json and case-insensitive word boundary replacement pipeline to resolve name pronunciation (like 'Aryan') and acronym spacing.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>configs/pronunciation_map.json, scripts/audio8/, voices/Social Media/that_feeling_of_being.wav, .venv/hf_cache/, D:\Saurav\TTS\workspace_history.xlsx</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
refactor: restructure TTS engine with new model test runners, unified voice assets, and project organization cleanup
</commit_message>
<xml_diff>
--- a/workspace_history.xlsx
+++ b/workspace_history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,24 +487,76 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Local Model Storage, Voice Sample Cleaning, Pronunciation Engine, &amp; UI Studio Enhancements</t>
+          <t>Local Model Storage, Voice Sample Cleaning, Pronunciation Engine, &amp; UI  Enhancements</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>1. Integrated Audio8-TTS-Preview-0.6b, a dual autoregressive multilingual zero-shot voice cloning model.
 2. Implemented custom transformers class registration mapping in scripts/audio8/ to resolve HuggingFace dynamic package import issues on Windows.
-3. Cleaned background noise from user MP3 voice sample using noisereduce, converted to WAV, transcribed with Whisper for naming (that_feeling_of_being.wav), and trimmed to 40.0s.
-4. Migrated HuggingFace weights cache (Kokoro, F5-TTS, Vocos, Whisper, Audio8) from global C: drive to local virtual environment (.venv/hf_cache) and set HF_HOME redirection.
-5. Filtered non-critical Python warnings (Google, Torchaudio, PyTorch) and muted HuggingFace HTTP HEAD connection retries in the console logs.
-6. Added interactive Voice Tuning post-processing sliders (Pitch shift, Speed/Tempo stretch, Audio Trimming) using librosa's phase vocoder.
-7. Designed the Voice Clone Arena comparison tab, enabling side-by-side prompt synthesis and latency metrics across multiple engines in columns.
-8. Createdconfigs/pronunciation_map.json and case-insensitive word boundary replacement pipeline to resolve name pronunciation (like 'Aryan') and acronym spacing.</t>
+3. Cleaned background noise from user MP3 voice sample using noisereduce, converted to WAV, transcribed with Whisper for naming (Sample.wav), and trimmed to 40.0s.
+4. Filtered non-critical Python warnings (Google, Torchaudio, PyTorch) and muted HuggingFace HTTP HEAD connection retries in the console logs.
+5. Added interactive Voice Tuning post-processing sliders (Pitch shift, Speed/Tempo stretch, Audio Trimming) using librosa's phase vocoder.
+6. Designed the Voice Clone Arena comparison tab, enabling side-by-side prompt synthesis and latency metrics across multiple engines in columns.
+7. Createdconfigs/pronunciation_map.json and case-insensitive word boundary replacement pipeline to resolve name pronunciation (like 'Aryan') and acronym spacing.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>configs/pronunciation_map.json, scripts/audio8/, voices/Social Media/that_feeling_of_being.wav, .venv/hf_cache/, D:\Saurav\TTS\workspace_history.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Voice Dataset Organization, GitHub Showcase &amp; HTML Lazy-Loading Architecture</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1. Sourced, cleaned, and organized 10 distinct voice profiles across 8 genres (Announcement, Audiobook, Motivational, Narration, Podcast, Presentation, Social Media, Storytelling).
+2. Processed voice samples using DeepFilterNet3, noisereduce, spectral subtraction, 80Hz high-pass filtering, and smooth cosine fade-ins/outs trimmed to &lt;=15s.
+3. Created batch synthesis engines (generate_all_model_samples.py &amp; build_new_models_folder.py) generating 90 voice samples across all 9 TTS models.
+4. Pushed 90 individual audio samples to GitHub repository (Aryan140314/Text-to-Speech-Models) using automated per-file commits.
+5. Re-architected TTS_Voice_Showcase.html to stream audio directly from GitHub raw URLs, reducing HTML size from 46MB down to 52KB for instant browser load times.
+6. Implemented interactive filter pills, search bar, and model tab navigation for seamless side-by-side voice comparison.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TTS_Voice_Showcase.html, models_all_voices/, push_to_github_one_by_one.py, build_new_models_folder.py, voices_clean/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Day 4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Context Overflow Auto-Chunking, Tokenizer Auto-Healing &amp; Structured Output Architecture</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1. Built _chunk_text_for_f5tts() sentence/clause splitter (300-word budget) with audio array concatenation to fix F5-TTS 8,192-token context limit errors.
+2. Implemented _clear_hf_model_cache() auto-healing to detect corrupted tokenizer.json files, wipe HF cache, and force clean re-downloads for Audio8.
+3. Added proactive multi-model stability guards: Chatterbox word length cap (500 words), Kokoro silent segment filtering (&lt;100 samples), and gTTS network timeout handling.
+4. Standardized output folder architecture (folder 1/) organizing 9 model subfolders ([ Model Name ]) with [Genre] VoiceName.wav output formatting.
+5. Produced voice_description_and_credits.md detailing voice source links, tone/pitch metrics, WPM pace, and 10,000-credit budget calculations.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>scripts/speech_synth_helper.py, D:\Saurav\TTS\1\, voice_description_and_credits.md, workspace_history.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>